<commit_message>
Add Fenix 6 spreadsheet
</commit_message>
<xml_diff>
--- a/sessions/paul/analysis/fenix-6-speeds.xlsx
+++ b/sessions/paul/analysis/fenix-6-speeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\mike\projects\docs\gps-guides\sessions\paul\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{587FB10D-8709-4AF5-8C80-00C9135C255B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35DC8F40-0428-4FB0-9B84-E7A3F5293EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440"/>
   </bookViews>
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -514,7 +514,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -588,31 +588,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>speed resolution (m)</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -652,17 +627,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'fenix-6-speeds'!$B$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>diff</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -675,522 +639,525 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>'fenix-6-speeds'!$B$2:$B$181</c:f>
+              <c:f>'fenix-6-speeds'!$B$4:$B$180</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="180"/>
+                <c:ptCount val="177"/>
+                <c:pt idx="0">
+                  <c:v>5.5999999999999994E-2</c:v>
+                </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.439</c:v>
+                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.5999999999999994E-2</c:v>
+                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.000000000000008E-3</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>2.8000000000000025E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
+                  <c:v>9.000000000000008E-3</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>2.8000000000000025E-2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.8000000000000025E-2</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
+                  <c:v>9.000000000000008E-3</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.9000000000000017E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="17">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="18">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
-                <c:pt idx="16">
-                  <c:v>9.000000000000008E-3</c:v>
-                </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
+                  <c:v>2.8000000000000025E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
                   <c:v>1.9000000000000017E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>2.8000000000000025E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.9000000000000017E-2</c:v>
+                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>2.8000000000000025E-2</c:v>
+                  <c:v>3.6999999999999922E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>9.000000000000008E-3</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>3.6999999999999922E-2</c:v>
+                  <c:v>1.8000000000000016E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.0000000000000009E-2</c:v>
+                  <c:v>3.8000000000000034E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>1.8000000000000016E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>3.8000000000000034E-2</c:v>
+                  <c:v>1.9000000000000017E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.8000000000000016E-2</c:v>
+                  <c:v>2.7999999999999914E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1.9000000000000017E-2</c:v>
+                  <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>2.7999999999999914E-2</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
                   <c:v>9.000000000000008E-3</c:v>
                 </c:pt>
                 <c:pt idx="33">
+                  <c:v>9.000000000000008E-3</c:v>
+                </c:pt>
+                <c:pt idx="34">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="34">
-                  <c:v>9.000000000000008E-3</c:v>
-                </c:pt>
                 <c:pt idx="35">
-                  <c:v>9.000000000000008E-3</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="36">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="37">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="37">
+                <c:pt idx="38">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="38">
+                <c:pt idx="39">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="39">
+                <c:pt idx="40">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="40">
+                <c:pt idx="41">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="41">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
                 <c:pt idx="42">
+                  <c:v>1.9000000000000128E-2</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>1.8000000000000016E-2</c:v>
+                </c:pt>
+                <c:pt idx="44">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="43">
+                <c:pt idx="45">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="44">
+                <c:pt idx="46">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="47">
                   <c:v>1.9000000000000128E-2</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>1.8000000000000016E-2</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="48">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>1.9000000000000128E-2</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="50">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="51">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="51">
+                <c:pt idx="52">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="52">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
                 <c:pt idx="53">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.8000000000000016E-2</c:v>
                 </c:pt>
                 <c:pt idx="54">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>1.8000000000000016E-2</c:v>
+                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="56">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="57">
                   <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="58">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="59">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="60">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="60">
+                <c:pt idx="61">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="61">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
                 <c:pt idx="62">
-                  <c:v>1.0000000000000009E-2</c:v>
+                  <c:v>1.9000000000000128E-2</c:v>
                 </c:pt>
                 <c:pt idx="63">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>1.9000000000000128E-2</c:v>
+                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="65">
+                  <c:v>1.0000000000000009E-2</c:v>
+                </c:pt>
+                <c:pt idx="66">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="66">
+                <c:pt idx="67">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="67">
+                <c:pt idx="68">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="68">
+                <c:pt idx="69">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="69">
+                <c:pt idx="70">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>1.0000000000000009E-2</c:v>
+                </c:pt>
+                <c:pt idx="72">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="70">
+                <c:pt idx="73">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="74">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="71">
+                <c:pt idx="75">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="76">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="72">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="73">
+                <c:pt idx="77">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="74">
+                <c:pt idx="78">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="75">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
                 <c:pt idx="79">
-                  <c:v>1.0000000000000009E-2</c:v>
+                  <c:v>1.8999999999999906E-2</c:v>
                 </c:pt>
                 <c:pt idx="80">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>1.8999999999999906E-2</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>9.000000000000119E-3</c:v>
+                  <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.8000000000000016E-2</c:v>
                 </c:pt>
                 <c:pt idx="84">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>1.8000000000000016E-2</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="86">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="87">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="87">
+                <c:pt idx="88">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="88">
+                <c:pt idx="89">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="89">
+                <c:pt idx="90">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="90">
+                <c:pt idx="91">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="91">
+                <c:pt idx="92">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="92">
+                <c:pt idx="93">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="93">
+                <c:pt idx="94">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="94">
+                <c:pt idx="95">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>1.0000000000000009E-2</c:v>
+                </c:pt>
+                <c:pt idx="97">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="95">
+                <c:pt idx="98">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="99">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="96">
+                <c:pt idx="100">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="101">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="97">
+                <c:pt idx="102">
+                  <c:v>1.0000000000000009E-2</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="104">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="98">
+                <c:pt idx="105">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="99">
+                <c:pt idx="106">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="100">
+                <c:pt idx="107">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="101">
+                <c:pt idx="108">
                   <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>8.999999999999897E-3</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="109">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="110">
-                  <c:v>1.0000000000000009E-2</c:v>
+                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="111">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="112">
+                  <c:v>1.0000000000000009E-2</c:v>
+                </c:pt>
+                <c:pt idx="113">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="113">
+                <c:pt idx="114">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="114">
+                <c:pt idx="115">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="115">
+                <c:pt idx="116">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="116">
+                <c:pt idx="117">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="117">
+                <c:pt idx="118">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="118">
+                <c:pt idx="119">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="119">
+                <c:pt idx="120">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="120">
+                <c:pt idx="121">
                   <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
                 <c:pt idx="122">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="123">
+                  <c:v>9.000000000000119E-3</c:v>
+                </c:pt>
+                <c:pt idx="124">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="124">
+                <c:pt idx="125">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="125">
+                <c:pt idx="126">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="126">
+                <c:pt idx="127">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="127">
+                <c:pt idx="128">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="128">
+                <c:pt idx="129">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="129">
+                <c:pt idx="130">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="130">
+                <c:pt idx="131">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="131">
+                <c:pt idx="132">
                   <c:v>9.000000000000119E-3</c:v>
                 </c:pt>
-                <c:pt idx="132">
+                <c:pt idx="133">
                   <c:v>1.0000000000000009E-2</c:v>
                 </c:pt>
-                <c:pt idx="133">
+                <c:pt idx="134">
+                  <c:v>8.9999999999996749E-3</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>9.0000000000003411E-3</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>9.9999999999997868E-3</c:v>
+                </c:pt>
+                <c:pt idx="137">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="134">
-                  <c:v>9.000000000000119E-3</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>1.0000000000000009E-2</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>8.9999999999996749E-3</c:v>
-                </c:pt>
-                <c:pt idx="137">
+                <c:pt idx="138">
                   <c:v>9.0000000000003411E-3</c:v>
                 </c:pt>
-                <c:pt idx="138">
+                <c:pt idx="139">
                   <c:v>9.9999999999997868E-3</c:v>
                 </c:pt>
-                <c:pt idx="139">
+                <c:pt idx="140">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="140">
+                <c:pt idx="141">
                   <c:v>9.0000000000003411E-3</c:v>
                 </c:pt>
-                <c:pt idx="141">
+                <c:pt idx="142">
                   <c:v>9.9999999999997868E-3</c:v>
                 </c:pt>
-                <c:pt idx="142">
+                <c:pt idx="143">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="143">
+                <c:pt idx="144">
                   <c:v>9.0000000000003411E-3</c:v>
                 </c:pt>
-                <c:pt idx="144">
+                <c:pt idx="145">
                   <c:v>9.9999999999997868E-3</c:v>
                 </c:pt>
-                <c:pt idx="145">
+                <c:pt idx="146">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
-                <c:pt idx="146">
-                  <c:v>9.0000000000003411E-3</c:v>
-                </c:pt>
                 <c:pt idx="147">
-                  <c:v>9.9999999999997868E-3</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="148">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.0000000000000231E-2</c:v>
                 </c:pt>
                 <c:pt idx="149">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="150">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="151">
                   <c:v>1.0000000000000231E-2</c:v>
-                </c:pt>
-                <c:pt idx="151">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="152">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="153">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="154">
                   <c:v>1.0000000000000231E-2</c:v>
-                </c:pt>
-                <c:pt idx="154">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="155">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="156">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="157">
                   <c:v>1.0000000000000231E-2</c:v>
-                </c:pt>
-                <c:pt idx="157">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="158">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="159">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="160">
                   <c:v>1.0000000000000231E-2</c:v>
-                </c:pt>
-                <c:pt idx="160">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="161">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="162">
+                  <c:v>8.999999999999897E-3</c:v>
+                </c:pt>
+                <c:pt idx="163">
                   <c:v>1.0000000000000231E-2</c:v>
-                </c:pt>
-                <c:pt idx="163">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="164">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="165">
-                  <c:v>1.0000000000000231E-2</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="166">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.9000000000000128E-2</c:v>
                 </c:pt>
                 <c:pt idx="167">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="168">
-                  <c:v>1.9000000000000128E-2</c:v>
+                  <c:v>1.0000000000000231E-2</c:v>
                 </c:pt>
                 <c:pt idx="169">
                   <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="170">
-                  <c:v>1.0000000000000231E-2</c:v>
+                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
                 <c:pt idx="171">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.9000000000000128E-2</c:v>
                 </c:pt>
                 <c:pt idx="172">
                   <c:v>8.999999999999897E-3</c:v>
@@ -1199,29 +1166,20 @@
                   <c:v>1.9000000000000128E-2</c:v>
                 </c:pt>
                 <c:pt idx="174">
-                  <c:v>8.999999999999897E-3</c:v>
+                  <c:v>1.8999999999999684E-2</c:v>
                 </c:pt>
                 <c:pt idx="175">
-                  <c:v>1.9000000000000128E-2</c:v>
+                  <c:v>9.0000000000003411E-3</c:v>
                 </c:pt>
                 <c:pt idx="176">
-                  <c:v>1.8999999999999684E-2</c:v>
-                </c:pt>
-                <c:pt idx="177">
-                  <c:v>9.0000000000003411E-3</c:v>
-                </c:pt>
-                <c:pt idx="178">
                   <c:v>2.8000000000000025E-2</c:v>
-                </c:pt>
-                <c:pt idx="179">
-                  <c:v>8.999999999999897E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BF51-4BF8-BA27-DC9DCAC39909}"/>
+              <c16:uniqueId val="{00000000-B50A-469D-A291-BB5CB00BFCD0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1235,11 +1193,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="552905104"/>
-        <c:axId val="552907400"/>
+        <c:axId val="430947472"/>
+        <c:axId val="430945176"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="552905104"/>
+        <c:axId val="430947472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1281,7 +1239,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="552907400"/>
+        <c:crossAx val="430945176"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1289,10 +1247,9 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="552907400"/>
+        <c:axId val="430945176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="0.1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1341,7 +1298,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="552905104"/>
+        <c:crossAx val="430947472"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1945,22 +1902,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>95249</xdr:rowOff>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>166</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>193</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A609F37-0F67-4451-9784-23C1A6887A73}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C2F1582-0C77-4558-93B1-88128AAEA69F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2299,17 +2256,14 @@
       <c r="A3" s="1">
         <v>0.439</v>
       </c>
-      <c r="B3" s="1">
-        <f>A3-A2</f>
-        <v>0.439</v>
-      </c>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>0.495</v>
       </c>
       <c r="B4" s="1">
-        <f>A4-A3</f>
+        <f t="shared" ref="B4:B67" si="0">A4-A3</f>
         <v>5.5999999999999994E-2</v>
       </c>
     </row>
@@ -2318,7 +2272,7 @@
         <v>0.504</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B68" si="0">A5-A4</f>
+        <f t="shared" si="0"/>
         <v>9.000000000000008E-3</v>
       </c>
     </row>
@@ -2885,7 +2839,7 @@
         <v>1.3340000000000001</v>
       </c>
       <c r="B68" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B68:B131" si="1">A68-A67</f>
         <v>9.000000000000119E-3</v>
       </c>
     </row>
@@ -2894,7 +2848,7 @@
         <v>1.3440000000000001</v>
       </c>
       <c r="B69" s="1">
-        <f t="shared" ref="B69:B132" si="1">A69-A68</f>
+        <f t="shared" si="1"/>
         <v>1.0000000000000009E-2</v>
       </c>
     </row>
@@ -3461,7 +3415,7 @@
         <v>1.95</v>
       </c>
       <c r="B132" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B132:B195" si="2">A132-A131</f>
         <v>8.999999999999897E-3</v>
       </c>
     </row>
@@ -3470,7 +3424,7 @@
         <v>1.9590000000000001</v>
       </c>
       <c r="B133" s="1">
-        <f t="shared" ref="B133:B196" si="2">A133-A132</f>
+        <f t="shared" si="2"/>
         <v>9.000000000000119E-3</v>
       </c>
     </row>
@@ -4037,7 +3991,7 @@
         <v>2.7149999999999999</v>
       </c>
       <c r="B196" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="B196:B259" si="3">A196-A195</f>
         <v>8.999999999999897E-3</v>
       </c>
     </row>
@@ -4046,7 +4000,7 @@
         <v>2.7250000000000001</v>
       </c>
       <c r="B197" s="1">
-        <f t="shared" ref="B197:B260" si="3">A197-A196</f>
+        <f t="shared" si="3"/>
         <v>1.0000000000000231E-2</v>
       </c>
     </row>
@@ -4613,7 +4567,7 @@
         <v>4.7770000000000001</v>
       </c>
       <c r="B260" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="B260:B323" si="4">A260-A259</f>
         <v>9.0000000000003411E-3</v>
       </c>
     </row>
@@ -4622,7 +4576,7 @@
         <v>4.7960000000000003</v>
       </c>
       <c r="B261" s="1">
-        <f t="shared" ref="B261:B324" si="4">A261-A260</f>
+        <f t="shared" si="4"/>
         <v>1.9000000000000128E-2</v>
       </c>
     </row>
@@ -5189,7 +5143,7 @@
         <v>5.944</v>
       </c>
       <c r="B324" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="B324:B387" si="5">A324-A323</f>
         <v>9.9999999999997868E-3</v>
       </c>
     </row>
@@ -5198,7 +5152,7 @@
         <v>5.9530000000000003</v>
       </c>
       <c r="B325" s="1">
-        <f t="shared" ref="B325:B388" si="5">A325-A324</f>
+        <f t="shared" si="5"/>
         <v>9.0000000000003411E-3</v>
       </c>
     </row>
@@ -5765,7 +5719,7 @@
         <v>6.9329999999999998</v>
       </c>
       <c r="B388" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="B388:B451" si="6">A388-A387</f>
         <v>1.9000000000000128E-2</v>
       </c>
     </row>
@@ -5774,7 +5728,7 @@
         <v>6.9420000000000002</v>
       </c>
       <c r="B389" s="1">
-        <f t="shared" ref="B389:B452" si="6">A389-A388</f>
+        <f t="shared" si="6"/>
         <v>9.0000000000003411E-3</v>
       </c>
     </row>
@@ -6341,7 +6295,7 @@
         <v>8.1739999999999995</v>
       </c>
       <c r="B452" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="B452:B515" si="7">A452-A451</f>
         <v>2.7999999999998693E-2</v>
       </c>
     </row>
@@ -6350,7 +6304,7 @@
         <v>8.1920000000000002</v>
       </c>
       <c r="B453" s="1">
-        <f t="shared" ref="B453:B516" si="7">A453-A452</f>
+        <f t="shared" si="7"/>
         <v>1.8000000000000682E-2</v>
       </c>
     </row>
@@ -6917,7 +6871,7 @@
         <v>9.7129999999999992</v>
       </c>
       <c r="B516" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="B516:B579" si="8">A516-A515</f>
         <v>8.9999999999985647E-3</v>
       </c>
     </row>
@@ -6926,7 +6880,7 @@
         <v>9.7319999999999993</v>
       </c>
       <c r="B517" s="1">
-        <f t="shared" ref="B517:B580" si="8">A517-A516</f>
+        <f t="shared" si="8"/>
         <v>1.9000000000000128E-2</v>
       </c>
     </row>
@@ -7493,7 +7447,7 @@
         <v>12.074</v>
       </c>
       <c r="B580" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="B580:B622" si="9">A580-A579</f>
         <v>9.0000000000003411E-3</v>
       </c>
     </row>
@@ -7502,7 +7456,7 @@
         <v>12.093</v>
       </c>
       <c r="B581" s="1">
-        <f t="shared" ref="B581:B622" si="9">A581-A580</f>
+        <f t="shared" si="9"/>
         <v>1.9000000000000128E-2</v>
       </c>
     </row>

</xml_diff>